<commit_message>
Log CI work; mark CI tasks done in the WBS
</commit_message>
<xml_diff>
--- a/docs/Project - WBS.xlsx
+++ b/docs/Project - WBS.xlsx
@@ -3255,7 +3255,7 @@
         <v>2.17</v>
       </c>
       <c r="J46" s="38" t="s">
-        <v>75</v>
+        <v>28</v>
       </c>
       <c r="K46" s="35">
         <f t="shared" ref="K46:K48" si="50">IF(J46="Done",1,IF(J46="In progress",0.5,0))</f>
@@ -3306,7 +3306,7 @@
         <v>2.17</v>
       </c>
       <c r="J47" s="38" t="s">
-        <v>75</v>
+        <v>28</v>
       </c>
       <c r="K47" s="35">
         <f t="shared" si="50"/>

</xml_diff>

<commit_message>
Move ticket side effects to events and queued listeners
</commit_message>
<xml_diff>
--- a/docs/Project - WBS.xlsx
+++ b/docs/Project - WBS.xlsx
@@ -3106,7 +3106,7 @@
         <v>2.17</v>
       </c>
       <c r="J43" s="38" t="s">
-        <v>75</v>
+        <v>28</v>
       </c>
       <c r="K43" s="35">
         <f t="shared" si="45"/>
@@ -3357,7 +3357,7 @@
         <v>2.17</v>
       </c>
       <c r="J48" s="38" t="s">
-        <v>75</v>
+        <v>28</v>
       </c>
       <c r="K48" s="35">
         <f t="shared" si="50"/>
@@ -3542,7 +3542,7 @@
         <v>2.17</v>
       </c>
       <c r="J52" s="38" t="s">
-        <v>75</v>
+        <v>28</v>
       </c>
       <c r="K52" s="35">
         <f t="shared" si="56"/>
@@ -3744,7 +3744,7 @@
         <v>2.17</v>
       </c>
       <c r="J56" s="38" t="s">
-        <v>75</v>
+        <v>28</v>
       </c>
       <c r="K56" s="35">
         <f t="shared" si="61"/>

</xml_diff>

<commit_message>
Add in-app notifications and notification bell
</commit_message>
<xml_diff>
--- a/docs/Project - WBS.xlsx
+++ b/docs/Project - WBS.xlsx
@@ -3892,10 +3892,8 @@
       <c r="I59" s="33">
         <v>3.25</v>
       </c>
-      <c r="J59" s="38" t="inlineStr">
-        <is>
-          <t>In progress</t>
-        </is>
+      <c r="J59" s="38" t="s">
+        <v>28</v>
       </c>
       <c r="K59" s="35">
         <f t="shared" ref="K59:K60" si="66">IF(J59="Done",1,IF(J59="In progress",0.5,0))</f>
@@ -3946,7 +3944,7 @@
         <v>3.25</v>
       </c>
       <c r="J60" s="38" t="s">
-        <v>75</v>
+        <v>28</v>
       </c>
       <c r="K60" s="35">
         <f t="shared" si="66"/>

</xml_diff>

<commit_message>
Add public REST API with Sanctum tokens, API resources, rate limiting and Scribe docs
</commit_message>
<xml_diff>
--- a/docs/Project - WBS.xlsx
+++ b/docs/Project - WBS.xlsx
@@ -4042,7 +4042,7 @@
         <v>2.17</v>
       </c>
       <c r="J62" s="38" t="s">
-        <v>75</v>
+        <v>28</v>
       </c>
       <c r="K62" s="35">
         <f t="shared" ref="K62:K64" si="70">IF(J62="Done",1,IF(J62="In progress",0.5,0))</f>
@@ -4093,7 +4093,7 @@
         <v>2.17</v>
       </c>
       <c r="J63" s="38" t="s">
-        <v>75</v>
+        <v>28</v>
       </c>
       <c r="K63" s="35">
         <f t="shared" si="70"/>
@@ -4144,7 +4144,7 @@
         <v>2.17</v>
       </c>
       <c r="J64" s="38" t="s">
-        <v>75</v>
+        <v>28</v>
       </c>
       <c r="K64" s="35">
         <f t="shared" si="70"/>
@@ -4241,10 +4241,8 @@
       <c r="I66" s="33">
         <v>2.17</v>
       </c>
-      <c r="J66" s="38" t="inlineStr">
-        <is>
-          <t>In progress</t>
-        </is>
+      <c r="J66" s="38" t="s">
+        <v>28</v>
       </c>
       <c r="K66" s="35">
         <f t="shared" ref="K66:K68" si="75">IF(J66="Done",1,IF(J66="In progress",0.5,0))</f>
@@ -4295,7 +4293,7 @@
         <v>2.17</v>
       </c>
       <c r="J67" s="38" t="s">
-        <v>75</v>
+        <v>28</v>
       </c>
       <c r="K67" s="35">
         <f t="shared" si="75"/>

</xml_diff>

<commit_message>
Run the queue on Laravel Horizon
</commit_message>
<xml_diff>
--- a/docs/Project - WBS.xlsx
+++ b/docs/Project - WBS.xlsx
@@ -3690,10 +3690,8 @@
       <c r="I55" s="33">
         <v>2.17</v>
       </c>
-      <c r="J55" s="38" t="inlineStr">
-        <is>
-          <t>In progress</t>
-        </is>
+      <c r="J55" s="38" t="s">
+        <v>28</v>
       </c>
       <c r="K55" s="35">
         <f t="shared" ref="K55:K57" si="61">IF(J55="Done",1,IF(J55="In progress",0.5,0))</f>

</xml_diff>

<commit_message>
Add Python FastAPI AI service with health and embed endpoints
</commit_message>
<xml_diff>
--- a/docs/Project - WBS.xlsx
+++ b/docs/Project - WBS.xlsx
@@ -4825,7 +4825,7 @@
         <v>2.17</v>
       </c>
       <c r="J78" s="38" t="s">
-        <v>75</v>
+        <v>28</v>
       </c>
       <c r="K78" s="35">
         <f t="shared" ref="K78:K80" si="90">IF(J78="Done",1,IF(J78="In progress",0.5,0))</f>
@@ -4876,7 +4876,7 @@
         <v>2.17</v>
       </c>
       <c r="J79" s="38" t="s">
-        <v>75</v>
+        <v>28</v>
       </c>
       <c r="K79" s="35">
         <f t="shared" si="90"/>
@@ -4927,7 +4927,7 @@
         <v>2.17</v>
       </c>
       <c r="J80" s="38" t="s">
-        <v>75</v>
+        <v>28</v>
       </c>
       <c r="K80" s="35">
         <f t="shared" si="90"/>
@@ -5024,8 +5024,10 @@
       <c r="I82" s="33">
         <v>2.17</v>
       </c>
-      <c r="J82" s="38" t="s">
-        <v>75</v>
+      <c r="J82" s="38" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
       </c>
       <c r="K82" s="35">
         <f t="shared" ref="K82:K84" si="95">IF(J82="Done",1,IF(J82="In progress",0.5,0))</f>
@@ -5075,8 +5077,10 @@
       <c r="I83" s="33">
         <v>2.17</v>
       </c>
-      <c r="J83" s="38" t="s">
-        <v>75</v>
+      <c r="J83" s="38" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
       </c>
       <c r="K83" s="35">
         <f t="shared" si="95"/>
@@ -5225,7 +5229,7 @@
         <v>2.17</v>
       </c>
       <c r="J86" s="38" t="s">
-        <v>75</v>
+        <v>28</v>
       </c>
       <c r="K86" s="35">
         <f t="shared" ref="K86:K88" si="100">IF(J86="Done",1,IF(J86="In progress",0.5,0))</f>
@@ -5276,7 +5280,7 @@
         <v>2.17</v>
       </c>
       <c r="J87" s="38" t="s">
-        <v>75</v>
+        <v>28</v>
       </c>
       <c r="K87" s="35">
         <f t="shared" si="100"/>

</xml_diff>

<commit_message>
Choose gemma3:1b as the local chat model (ADR-003) and add chat to the AI service
</commit_message>
<xml_diff>
--- a/docs/Project - WBS.xlsx
+++ b/docs/Project - WBS.xlsx
@@ -5024,10 +5024,8 @@
       <c r="I82" s="33">
         <v>2.17</v>
       </c>
-      <c r="J82" s="38" t="inlineStr">
-        <is>
-          <t>In progress</t>
-        </is>
+      <c r="J82" s="38" t="s">
+        <v>28</v>
       </c>
       <c r="K82" s="35">
         <f t="shared" ref="K82:K84" si="95">IF(J82="Done",1,IF(J82="In progress",0.5,0))</f>
@@ -5077,10 +5075,8 @@
       <c r="I83" s="33">
         <v>2.17</v>
       </c>
-      <c r="J83" s="38" t="inlineStr">
-        <is>
-          <t>In progress</t>
-        </is>
+      <c r="J83" s="38" t="s">
+        <v>28</v>
       </c>
       <c r="K83" s="35">
         <f t="shared" si="95"/>
@@ -5131,7 +5127,7 @@
         <v>2.17</v>
       </c>
       <c r="J84" s="38" t="s">
-        <v>75</v>
+        <v>28</v>
       </c>
       <c r="K84" s="35">
         <f t="shared" si="95"/>

</xml_diff>

<commit_message>
Add AI-suggested replies from the knowledge base (RAG) and a project guide
</commit_message>
<xml_diff>
--- a/docs/Project - WBS.xlsx
+++ b/docs/Project - WBS.xlsx
@@ -5661,7 +5661,7 @@
         <v>3.25</v>
       </c>
       <c r="J95" s="38" t="s">
-        <v>75</v>
+        <v>28</v>
       </c>
       <c r="K95" s="35">
         <f t="shared" ref="K95:K96" si="111">IF(J95="Done",1,IF(J95="In progress",0.5,0))</f>
@@ -5712,7 +5712,7 @@
         <v>3.25</v>
       </c>
       <c r="J96" s="38" t="s">
-        <v>75</v>
+        <v>28</v>
       </c>
       <c r="K96" s="35">
         <f t="shared" si="111"/>

</xml_diff>